<commit_message>
Indicators results updates and xls files added
</commit_message>
<xml_diff>
--- a/InitializationResults/WithTrack/Comparison of NSGAII with NSGAII_SI for each generation (on average).xlsx
+++ b/InitializationResults/WithTrack/Comparison of NSGAII with NSGAII_SI for each generation (on average).xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10995" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10995"/>
   </bookViews>
   <sheets>
     <sheet name="EPS" sheetId="1" r:id="rId1"/>
@@ -71,10 +71,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -107,6 +107,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="it-IT"/>
+              <a:t>Epsilon</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
@@ -141,14 +166,19 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
+        <c:scatterStyle val="smoothMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>NSGAII</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
-              <a:noFill/>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -606,14 +636,19 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>NSGAII_SI</c:v>
+          </c:tx>
           <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -852,7 +887,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -862,11 +897,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="378599456"/>
-        <c:axId val="378606904"/>
+        <c:axId val="233025784"/>
+        <c:axId val="233030096"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="378599456"/>
+        <c:axId val="233025784"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -886,6 +921,62 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>Generation</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="it-IT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -923,12 +1014,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="378606904"/>
+        <c:crossAx val="233030096"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="378606904"/>
+        <c:axId val="233030096"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -985,7 +1076,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="378599456"/>
+        <c:crossAx val="233025784"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -997,6 +1088,38 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -1049,6 +1172,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="it-IT"/>
+              <a:t>Generational Distance (GD)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
@@ -1083,14 +1231,19 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
+        <c:scatterStyle val="smoothMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>NSGAII</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
-              <a:noFill/>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -1548,14 +1701,19 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>NSGAII_SI</c:v>
+          </c:tx>
           <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -1794,7 +1952,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -1804,11 +1962,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="510494328"/>
-        <c:axId val="510493152"/>
+        <c:axId val="233034408"/>
+        <c:axId val="233027352"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="510494328"/>
+        <c:axId val="233034408"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1828,6 +1986,62 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>Generation</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="it-IT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1865,12 +2079,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="510493152"/>
+        <c:crossAx val="233027352"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="510493152"/>
+        <c:axId val="233027352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1927,7 +2141,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="510494328"/>
+        <c:crossAx val="233034408"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1939,6 +2153,38 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -1991,6 +2237,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="it-IT"/>
+              <a:t>Hypervolume</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
@@ -2025,14 +2296,19 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
+        <c:scatterStyle val="smoothMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>NSGAII</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
-              <a:noFill/>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -2490,14 +2766,19 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>NSGAII_SI</c:v>
+          </c:tx>
           <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -2736,7 +3017,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -2746,11 +3027,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="378602984"/>
-        <c:axId val="378602592"/>
+        <c:axId val="233033232"/>
+        <c:axId val="233026176"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="378602984"/>
+        <c:axId val="233033232"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2770,6 +3051,62 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>Generation</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="it-IT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -2807,12 +3144,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="378602592"/>
+        <c:crossAx val="233026176"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="378602592"/>
+        <c:axId val="233026176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0.65000000000000013"/>
@@ -2870,7 +3207,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="378602984"/>
+        <c:crossAx val="233033232"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2882,6 +3219,38 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -2934,6 +3303,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="it-IT"/>
+              <a:t>Inverted Generational Distance (IGD)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
@@ -2968,14 +3362,19 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
+        <c:scatterStyle val="smoothMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>NSGAII</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
-              <a:noFill/>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -3433,14 +3832,19 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>NSGAII_SI</c:v>
+          </c:tx>
           <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -3679,7 +4083,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -3689,11 +4093,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="514295360"/>
-        <c:axId val="514294576"/>
+        <c:axId val="233035192"/>
+        <c:axId val="233024216"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="514295360"/>
+        <c:axId val="233035192"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3713,6 +4117,62 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>Generation</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="it-IT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -3750,12 +4210,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="514294576"/>
+        <c:crossAx val="233024216"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="514294576"/>
+        <c:axId val="233024216"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3812,7 +4272,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="514295360"/>
+        <c:crossAx val="233035192"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3824,6 +4284,38 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -3876,6 +4368,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="it-IT"/>
+              <a:t>Spread</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
@@ -3910,14 +4427,19 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
+        <c:scatterStyle val="smoothMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>NSGAII</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
-              <a:noFill/>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -4375,14 +4897,19 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>NSGAII_SI</c:v>
+          </c:tx>
           <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -4621,7 +5148,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -4631,11 +5158,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="508941704"/>
-        <c:axId val="508941312"/>
+        <c:axId val="233039112"/>
+        <c:axId val="233037936"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="508941704"/>
+        <c:axId val="233039112"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4655,6 +5182,62 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>Generation</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="it-IT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -4692,12 +5275,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="508941312"/>
+        <c:crossAx val="233037936"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="508941312"/>
+        <c:axId val="233037936"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4754,7 +5337,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="508941704"/>
+        <c:crossAx val="233039112"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4766,6 +5349,38 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -7587,16 +8202,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>200025</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>428625</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>90487</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7615,6 +8230,725 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6157914" cy="1171576"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="3" name="TextBox 2"/>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="2733675" y="190500"/>
+              <a:ext cx="6157914" cy="1171576"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:noAutofit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑖𝑛</m:t>
+                    </m:r>
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑑</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑖</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>= </m:t>
+                    </m:r>
+                    <m:f>
+                      <m:fPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:fPr>
+                      <m:num>
+                        <m:nary>
+                          <m:naryPr>
+                            <m:chr m:val="∑"/>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:naryPr>
+                          <m:sub>
+                            <m:r>
+                              <m:rPr>
+                                <m:brk m:alnAt="23"/>
+                              </m:rPr>
+                              <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑗</m:t>
+                            </m:r>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>=1</m:t>
+                            </m:r>
+                          </m:sub>
+                          <m:sup>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑛𝑟</m:t>
+                            </m:r>
+                          </m:sup>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑖𝑛</m:t>
+                            </m:r>
+                            <m:sSub>
+                              <m:sSubPr>
+                                <m:ctrlPr>
+                                  <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                  </a:rPr>
+                                </m:ctrlPr>
+                              </m:sSubPr>
+                              <m:e>
+                                <m:r>
+                                  <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                  </a:rPr>
+                                  <m:t>𝑑</m:t>
+                                </m:r>
+                              </m:e>
+                              <m:sub>
+                                <m:r>
+                                  <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                                  </a:rPr>
+                                  <m:t>𝑖𝑗</m:t>
+                                </m:r>
+                              </m:sub>
+                            </m:sSub>
+                          </m:e>
+                        </m:nary>
+                      </m:num>
+                      <m:den>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑛𝑟</m:t>
+                        </m:r>
+                      </m:den>
+                    </m:f>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="it-IT" sz="1400"/>
+            </a:p>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑖𝑛</m:t>
+                    </m:r>
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑑</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑖</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑖𝑠</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑡h𝑒</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑖𝑛𝑑𝑖𝑐𝑎𝑡𝑜𝑟</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑣𝑎𝑙𝑢𝑒</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑓𝑜𝑟</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:sSup>
+                      <m:sSupPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSupPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑖</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sup>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑡h</m:t>
+                        </m:r>
+                      </m:sup>
+                    </m:sSup>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑔𝑒𝑛𝑒𝑟𝑎𝑡𝑖𝑜</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>, </m:t>
+                    </m:r>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="en-US" sz="1400" b="0" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑛𝑟</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑖𝑠</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑡h𝑒</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑛𝑢𝑚𝑏𝑒𝑟</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑜𝑓</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑟𝑒𝑝𝑒𝑎𝑡𝑖𝑜𝑛</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑜𝑟</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑟𝑢𝑛𝑠</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>, </m:t>
+                    </m:r>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="en-US" sz="1400" b="0" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑖𝑛</m:t>
+                    </m:r>
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑑</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑖𝑗</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t> </m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑖𝑠</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑡h𝑒</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑖𝑛𝑑𝑖𝑐𝑎𝑡𝑜𝑟</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑣𝑎𝑙𝑢𝑒</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑜𝑓</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:sSup>
+                      <m:sSupPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSupPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑖</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sup>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑡h</m:t>
+                        </m:r>
+                      </m:sup>
+                    </m:sSup>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑔𝑒𝑛𝑒𝑟𝑎𝑡𝑖𝑜𝑛</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑜𝑓</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:sSup>
+                      <m:sSupPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSupPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑗</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sup>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑡h</m:t>
+                        </m:r>
+                      </m:sup>
+                    </m:sSup>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>𝑟𝑢𝑛</m:t>
+                    </m:r>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="en-US" sz="1400" b="0"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="3" name="TextBox 2"/>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="2733675" y="190500"/>
+              <a:ext cx="6157914" cy="1171576"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:noAutofit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="en-US" sz="1400" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑖𝑛𝑑_𝑖=  (∑_(𝑗=1)^𝑛𝑟▒〖𝑖𝑛𝑑_𝑖𝑗 〗)/𝑛𝑟</a:t>
+              </a:r>
+              <a:endParaRPr lang="it-IT" sz="1400"/>
+            </a:p>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="en-US" sz="1400" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑖𝑛𝑑_𝑖  𝑖𝑠 𝑡ℎ𝑒 𝑖𝑛𝑑𝑖𝑐𝑎𝑡𝑜𝑟 𝑣𝑎𝑙𝑢𝑒 𝑓𝑜𝑟 𝑖^𝑡ℎ 𝑔𝑒𝑛𝑒𝑟𝑎𝑡𝑖𝑜, </a:t>
+              </a:r>
+              <a:endParaRPr lang="en-US" sz="1400" b="0" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="en-US" sz="1400" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑛𝑟 𝑖𝑠 𝑡ℎ𝑒 𝑛𝑢𝑚𝑏𝑒𝑟 𝑜𝑓 𝑟𝑒𝑝𝑒𝑎𝑡𝑖𝑜𝑛 𝑜𝑟 𝑟𝑢𝑛𝑠, </a:t>
+              </a:r>
+              <a:endParaRPr lang="en-US" sz="1400" b="0" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="en-US" sz="1400" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑖𝑛𝑑_(𝑖𝑗 ) 𝑖𝑠 𝑡ℎ𝑒 𝑖𝑛𝑑𝑖𝑐𝑎𝑡𝑜𝑟 𝑣𝑎𝑙𝑢𝑒 𝑜𝑓 𝑖^𝑡ℎ 𝑔𝑒𝑛𝑒𝑟𝑎𝑡𝑖𝑜𝑛 𝑜𝑓 𝑗^𝑡ℎ 𝑟𝑢𝑛</a:t>
+              </a:r>
+              <a:endParaRPr lang="en-US" sz="1400" b="0"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -7622,16 +8956,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>333375</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>428625</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>90487</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7657,16 +8991,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>428625</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>90487</xdr:rowOff>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>119062</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7692,16 +9026,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>428625</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>90487</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>185737</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7727,16 +9061,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>428625</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>90487</xdr:rowOff>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>33337</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8025,14 +9359,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -9030,14 +10364,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -9231,7 +10565,7 @@
       <c r="C15">
         <v>14</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>9.0883116938525303E-4</v>
       </c>
     </row>
@@ -9239,13 +10573,13 @@
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="1">
         <v>9.2253163283763796E-4</v>
       </c>
       <c r="C16">
         <v>15</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>8.3438221475302097E-4</v>
       </c>
     </row>
@@ -9253,13 +10587,13 @@
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <v>8.47669526110021E-4</v>
       </c>
       <c r="C17">
         <v>16</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>7.80675983803895E-4</v>
       </c>
     </row>
@@ -9267,13 +10601,13 @@
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <v>7.9150650370939601E-4</v>
       </c>
       <c r="C18">
         <v>17</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>7.2276514432390395E-4</v>
       </c>
     </row>
@@ -9281,13 +10615,13 @@
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="1">
         <v>7.48181500298473E-4</v>
       </c>
       <c r="C19">
         <v>18</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>6.9008205560913997E-4</v>
       </c>
     </row>
@@ -9295,13 +10629,13 @@
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="1">
         <v>7.1114687764625695E-4</v>
       </c>
       <c r="C20">
         <v>19</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>6.5433151134782397E-4</v>
       </c>
     </row>
@@ -9309,13 +10643,13 @@
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="1">
         <v>6.6228085214212803E-4</v>
       </c>
       <c r="C21">
         <v>20</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>6.1155745660518095E-4</v>
       </c>
     </row>
@@ -9323,13 +10657,13 @@
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="1">
         <v>6.2125290056156996E-4</v>
       </c>
       <c r="C22">
         <v>21</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>5.7418792124796895E-4</v>
       </c>
     </row>
@@ -9337,13 +10671,13 @@
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="1">
         <v>5.6890341188297103E-4</v>
       </c>
       <c r="C23">
         <v>22</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>5.3080696486497198E-4</v>
       </c>
     </row>
@@ -9351,13 +10685,13 @@
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="1">
         <v>5.4779069296664602E-4</v>
       </c>
       <c r="C24">
         <v>23</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="1">
         <v>5.1688082885305395E-4</v>
       </c>
     </row>
@@ -9365,13 +10699,13 @@
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="1">
         <v>5.1802121603684295E-4</v>
       </c>
       <c r="C25">
         <v>24</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="1">
         <v>4.9627885904685997E-4</v>
       </c>
     </row>
@@ -9379,13 +10713,13 @@
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="1">
         <v>4.8499376756276001E-4</v>
       </c>
       <c r="C26">
         <v>25</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>4.7774379937558898E-4</v>
       </c>
     </row>
@@ -9393,13 +10727,13 @@
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27" s="1">
         <v>4.6879331197938098E-4</v>
       </c>
       <c r="C27">
         <v>26</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>4.6897708181837801E-4</v>
       </c>
     </row>
@@ -9407,13 +10741,13 @@
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="1">
         <v>4.57283968382422E-4</v>
       </c>
       <c r="C28">
         <v>27</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>4.6344539457096601E-4</v>
       </c>
     </row>
@@ -9421,13 +10755,13 @@
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="1">
         <v>4.24900547165198E-4</v>
       </c>
       <c r="C29">
         <v>28</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>4.5712133385636899E-4</v>
       </c>
     </row>
@@ -9435,13 +10769,13 @@
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="1">
         <v>4.20908913669575E-4</v>
       </c>
       <c r="C30">
         <v>29</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>4.4714806172369302E-4</v>
       </c>
     </row>
@@ -9449,13 +10783,13 @@
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="1">
         <v>4.05614331960135E-4</v>
       </c>
       <c r="C31">
         <v>30</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>4.3424867606708999E-4</v>
       </c>
     </row>
@@ -9463,13 +10797,13 @@
       <c r="A32">
         <v>31</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="1">
         <v>3.8480583313421402E-4</v>
       </c>
       <c r="C32">
         <v>31</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D32" s="1">
         <v>4.1990890500149299E-4</v>
       </c>
     </row>
@@ -9477,13 +10811,13 @@
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="1">
         <v>3.68814584498239E-4</v>
       </c>
       <c r="C33">
         <v>32</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>4.08127887148878E-4</v>
       </c>
     </row>
@@ -9491,13 +10825,13 @@
       <c r="A34">
         <v>33</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34" s="1">
         <v>3.5787141233278999E-4</v>
       </c>
       <c r="C34">
         <v>33</v>
       </c>
-      <c r="D34" s="2">
+      <c r="D34" s="1">
         <v>3.9949651889824203E-4</v>
       </c>
     </row>
@@ -9505,13 +10839,13 @@
       <c r="A35">
         <v>34</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="1">
         <v>3.5082951848556501E-4</v>
       </c>
       <c r="C35">
         <v>34</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>4.01170572958099E-4</v>
       </c>
     </row>
@@ -9519,13 +10853,13 @@
       <c r="A36">
         <v>35</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B36" s="1">
         <v>3.5102780908237901E-4</v>
       </c>
       <c r="C36">
         <v>35</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>4.0429476296078399E-4</v>
       </c>
     </row>
@@ -9533,13 +10867,13 @@
       <c r="A37">
         <v>36</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37" s="1">
         <v>3.4800927330132703E-4</v>
       </c>
       <c r="C37">
         <v>36</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>4.1313147620511902E-4</v>
       </c>
     </row>
@@ -9547,13 +10881,13 @@
       <c r="A38">
         <v>37</v>
       </c>
-      <c r="B38" s="2">
+      <c r="B38" s="1">
         <v>3.5367302098830602E-4</v>
       </c>
       <c r="C38">
         <v>37</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>4.1239352929854802E-4</v>
       </c>
     </row>
@@ -9561,13 +10895,13 @@
       <c r="A39">
         <v>38</v>
       </c>
-      <c r="B39" s="2">
+      <c r="B39" s="1">
         <v>3.4944995019321398E-4</v>
       </c>
       <c r="C39">
         <v>38</v>
       </c>
-      <c r="D39" s="2">
+      <c r="D39" s="1">
         <v>4.1656672140509901E-4</v>
       </c>
     </row>
@@ -9575,13 +10909,13 @@
       <c r="A40">
         <v>39</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B40" s="1">
         <v>3.5658767991817298E-4</v>
       </c>
       <c r="C40">
         <v>39</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>3.9622777619184498E-4</v>
       </c>
     </row>
@@ -9589,13 +10923,13 @@
       <c r="A41">
         <v>40</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41" s="1">
         <v>3.5012071970403502E-4</v>
       </c>
       <c r="C41">
         <v>40</v>
       </c>
-      <c r="D41" s="2">
+      <c r="D41" s="1">
         <v>3.9097798132477598E-4</v>
       </c>
     </row>
@@ -9603,13 +10937,13 @@
       <c r="A42">
         <v>41</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="1">
         <v>3.3646307805431801E-4</v>
       </c>
       <c r="C42">
         <v>41</v>
       </c>
-      <c r="D42" s="2">
+      <c r="D42" s="1">
         <v>4.0155308482939201E-4</v>
       </c>
     </row>
@@ -9617,13 +10951,13 @@
       <c r="A43">
         <v>42</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="1">
         <v>3.3880208589706298E-4</v>
       </c>
       <c r="C43">
         <v>42</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>3.95903884011385E-4</v>
       </c>
     </row>
@@ -9631,13 +10965,13 @@
       <c r="A44">
         <v>43</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>3.3657289854348402E-4</v>
       </c>
       <c r="C44">
         <v>43</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>3.9830389304178898E-4</v>
       </c>
     </row>
@@ -9645,13 +10979,13 @@
       <c r="A45">
         <v>44</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="1">
         <v>3.38396341422133E-4</v>
       </c>
       <c r="C45">
         <v>44</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>3.9288132404300498E-4</v>
       </c>
     </row>
@@ -9659,13 +10993,13 @@
       <c r="A46">
         <v>45</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="1">
         <v>3.4086490485094999E-4</v>
       </c>
       <c r="C46">
         <v>45</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>3.9927963442358099E-4</v>
       </c>
     </row>
@@ -9673,13 +11007,13 @@
       <c r="A47">
         <v>46</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47" s="1">
         <v>3.31339641448088E-4</v>
       </c>
       <c r="C47">
         <v>46</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>3.8739548534710399E-4</v>
       </c>
     </row>
@@ -9687,13 +11021,13 @@
       <c r="A48">
         <v>47</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48" s="1">
         <v>3.1979769174208698E-4</v>
       </c>
       <c r="C48">
         <v>47</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>3.91261413778322E-4</v>
       </c>
     </row>
@@ -9701,13 +11035,13 @@
       <c r="A49">
         <v>48</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49" s="1">
         <v>3.1633147739676501E-4</v>
       </c>
       <c r="C49">
         <v>48</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>3.9451120698353801E-4</v>
       </c>
     </row>
@@ -9715,13 +11049,13 @@
       <c r="A50">
         <v>49</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="1">
         <v>3.1904142562728997E-4</v>
       </c>
       <c r="C50">
         <v>49</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>3.9038156859295199E-4</v>
       </c>
     </row>
@@ -9729,13 +11063,13 @@
       <c r="A51">
         <v>50</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B51" s="1">
         <v>3.1524407852689002E-4</v>
       </c>
       <c r="C51">
         <v>50</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>3.8622455702593401E-4</v>
       </c>
     </row>
@@ -9743,13 +11077,13 @@
       <c r="A52">
         <v>51</v>
       </c>
-      <c r="B52" s="2">
+      <c r="B52" s="1">
         <v>3.1398976210366601E-4</v>
       </c>
       <c r="C52">
         <v>51</v>
       </c>
-      <c r="D52" s="2">
+      <c r="D52" s="1">
         <v>3.8946630727969901E-4</v>
       </c>
     </row>
@@ -9757,13 +11091,13 @@
       <c r="A53">
         <v>52</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="1">
         <v>3.1228635063619E-4</v>
       </c>
       <c r="C53">
         <v>52</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>3.7631392000020701E-4</v>
       </c>
     </row>
@@ -9771,13 +11105,13 @@
       <c r="A54">
         <v>53</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="1">
         <v>3.1621012869359499E-4</v>
       </c>
       <c r="C54">
         <v>53</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>3.7719577190108898E-4</v>
       </c>
     </row>
@@ -9785,13 +11119,13 @@
       <c r="A55">
         <v>54</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55" s="1">
         <v>3.0798713378064901E-4</v>
       </c>
       <c r="C55">
         <v>54</v>
       </c>
-      <c r="D55" s="2">
+      <c r="D55" s="1">
         <v>3.8028280381384802E-4</v>
       </c>
     </row>
@@ -9799,13 +11133,13 @@
       <c r="A56">
         <v>55</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B56" s="1">
         <v>3.16211758354541E-4</v>
       </c>
       <c r="C56">
         <v>55</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>3.8233539870019198E-4</v>
       </c>
     </row>
@@ -9813,13 +11147,13 @@
       <c r="A57">
         <v>56</v>
       </c>
-      <c r="B57" s="2">
+      <c r="B57" s="1">
         <v>3.1279779739524702E-4</v>
       </c>
       <c r="C57">
         <v>56</v>
       </c>
-      <c r="D57" s="2">
+      <c r="D57" s="1">
         <v>3.8383433552139002E-4</v>
       </c>
     </row>
@@ -9827,13 +11161,13 @@
       <c r="A58">
         <v>57</v>
       </c>
-      <c r="B58" s="2">
+      <c r="B58" s="1">
         <v>3.12885506473467E-4</v>
       </c>
       <c r="C58">
         <v>57</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>3.8097738739993901E-4</v>
       </c>
     </row>
@@ -9841,13 +11175,13 @@
       <c r="A59">
         <v>58</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="1">
         <v>3.1140773317617503E-4</v>
       </c>
       <c r="C59">
         <v>58</v>
       </c>
-      <c r="D59" s="2">
+      <c r="D59" s="1">
         <v>3.8222149940857902E-4</v>
       </c>
     </row>
@@ -9855,13 +11189,13 @@
       <c r="A60">
         <v>59</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="1">
         <v>3.1206531355423199E-4</v>
       </c>
       <c r="C60">
         <v>59</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>3.78760028931395E-4</v>
       </c>
     </row>
@@ -9869,13 +11203,13 @@
       <c r="A61">
         <v>60</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="1">
         <v>3.1623898762415102E-4</v>
       </c>
       <c r="C61">
         <v>60</v>
       </c>
-      <c r="D61" s="2">
+      <c r="D61" s="1">
         <v>3.7455425911435598E-4</v>
       </c>
     </row>
@@ -9883,13 +11217,13 @@
       <c r="A62">
         <v>61</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B62" s="1">
         <v>3.0798550473855102E-4</v>
       </c>
       <c r="C62">
         <v>61</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>3.7072332230313697E-4</v>
       </c>
     </row>
@@ -9897,13 +11231,13 @@
       <c r="A63">
         <v>62</v>
       </c>
-      <c r="B63" s="2">
+      <c r="B63" s="1">
         <v>3.08075534056743E-4</v>
       </c>
       <c r="C63">
         <v>62</v>
       </c>
-      <c r="D63" s="2">
+      <c r="D63" s="1">
         <v>3.6316677801223601E-4</v>
       </c>
     </row>
@@ -9911,13 +11245,13 @@
       <c r="A64">
         <v>63</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="1">
         <v>3.04940745985122E-4</v>
       </c>
       <c r="C64">
         <v>63</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>3.5427950006193803E-4</v>
       </c>
     </row>
@@ -9925,13 +11259,13 @@
       <c r="A65">
         <v>64</v>
       </c>
-      <c r="B65" s="2">
+      <c r="B65" s="1">
         <v>3.0519287959425098E-4</v>
       </c>
       <c r="C65">
         <v>64</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>3.5098998913497299E-4</v>
       </c>
     </row>
@@ -9939,13 +11273,13 @@
       <c r="A66">
         <v>65</v>
       </c>
-      <c r="B66" s="2">
+      <c r="B66" s="1">
         <v>3.12792705353473E-4</v>
       </c>
       <c r="C66">
         <v>65</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>3.4879522474423499E-4</v>
       </c>
     </row>
@@ -9953,13 +11287,13 @@
       <c r="A67">
         <v>66</v>
       </c>
-      <c r="B67" s="2">
+      <c r="B67" s="1">
         <v>3.0113278074980299E-4</v>
       </c>
       <c r="C67">
         <v>66</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>3.6394457758151701E-4</v>
       </c>
     </row>
@@ -9967,13 +11301,13 @@
       <c r="A68">
         <v>67</v>
       </c>
-      <c r="B68" s="2">
+      <c r="B68" s="1">
         <v>3.0180922307701698E-4</v>
       </c>
       <c r="C68">
         <v>67</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>3.5337792221981401E-4</v>
       </c>
     </row>
@@ -9981,13 +11315,13 @@
       <c r="A69">
         <v>68</v>
       </c>
-      <c r="B69" s="2">
+      <c r="B69" s="1">
         <v>2.9598180197460902E-4</v>
       </c>
       <c r="C69">
         <v>68</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>3.4898961428167502E-4</v>
       </c>
     </row>
@@ -9995,13 +11329,13 @@
       <c r="A70">
         <v>69</v>
       </c>
-      <c r="B70" s="2">
+      <c r="B70" s="1">
         <v>2.9677232784032102E-4</v>
       </c>
       <c r="C70">
         <v>69</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>3.4365049754743297E-4</v>
       </c>
     </row>
@@ -10009,13 +11343,13 @@
       <c r="A71">
         <v>70</v>
       </c>
-      <c r="B71" s="2">
+      <c r="B71" s="1">
         <v>2.9019498285911302E-4</v>
       </c>
       <c r="C71">
         <v>70</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>3.45993353399636E-4</v>
       </c>
     </row>
@@ -10035,14 +11369,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -11040,14 +12374,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -12045,14 +13379,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">

</xml_diff>

<commit_message>
Results with tracking (indicator values for each generation) for initialization are updated
</commit_message>
<xml_diff>
--- a/InitializationResults/WithTrack/Comparison of NSGAII with NSGAII_SI for each generation (on average).xlsx
+++ b/InitializationResults/WithTrack/Comparison of NSGAII with NSGAII_SI for each generation (on average).xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10995" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10995"/>
   </bookViews>
   <sheets>
     <sheet name="EPS" sheetId="1" r:id="rId1"/>
@@ -897,11 +897,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="346524912"/>
-        <c:axId val="346532360"/>
+        <c:axId val="356932088"/>
+        <c:axId val="356929344"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="346524912"/>
+        <c:axId val="356932088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1014,12 +1014,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346532360"/>
+        <c:crossAx val="356929344"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="346532360"/>
+        <c:axId val="356929344"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1076,7 +1076,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346524912"/>
+        <c:crossAx val="356932088"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1962,11 +1962,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="346527656"/>
-        <c:axId val="346525304"/>
+        <c:axId val="356932480"/>
+        <c:axId val="356930128"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="346527656"/>
+        <c:axId val="356932480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2079,12 +2079,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346525304"/>
+        <c:crossAx val="356930128"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="346525304"/>
+        <c:axId val="356930128"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2141,7 +2141,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346527656"/>
+        <c:crossAx val="356932480"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3027,11 +3027,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="346530792"/>
-        <c:axId val="346523736"/>
+        <c:axId val="356930912"/>
+        <c:axId val="360335112"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="346530792"/>
+        <c:axId val="356930912"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3144,12 +3144,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346523736"/>
+        <c:crossAx val="360335112"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="346523736"/>
+        <c:axId val="360335112"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0.65000000000000013"/>
@@ -3207,7 +3207,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346530792"/>
+        <c:crossAx val="356930912"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4093,11 +4093,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="346531576"/>
-        <c:axId val="346525696"/>
+        <c:axId val="360337464"/>
+        <c:axId val="360338248"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="346531576"/>
+        <c:axId val="360337464"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4210,12 +4210,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346525696"/>
+        <c:crossAx val="360338248"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="346525696"/>
+        <c:axId val="360338248"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4272,7 +4272,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346531576"/>
+        <c:crossAx val="360337464"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5158,11 +5158,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="346522560"/>
-        <c:axId val="346526872"/>
+        <c:axId val="360335504"/>
+        <c:axId val="360337856"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="346522560"/>
+        <c:axId val="360335504"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5275,12 +5275,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346526872"/>
+        <c:crossAx val="360337856"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="346526872"/>
+        <c:axId val="360337856"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5337,7 +5337,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346522560"/>
+        <c:crossAx val="360335504"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>

</xml_diff>